<commit_message>
Add PROM adapter components to parts list
</commit_message>
<xml_diff>
--- a/inboard386/parts_list.xlsx
+++ b/inboard386/parts_list.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="154">
   <si>
     <t xml:space="preserve">Part:</t>
   </si>
@@ -428,6 +428,69 @@
   </si>
   <si>
     <t xml:space="preserve">3365/40-CUT-LENGTH</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">--------------------- </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">PROM adapter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> ---------------------</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">EEPROM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">556-AT28HC64B90JU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AT28HC64B-90JU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27C512 pin compatible and 120ns or faster</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLCC32 socket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">737-PLCC-32-AT-SMT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLCC-32-AT-SMT</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 595-SN74F32DRE4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SN74F32DRE4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">581-KAM21BR71H104JT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAM21BR71H104JT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PinHeader 1x10</t>
   </si>
   <si>
     <r>
@@ -727,7 +790,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.97"/>
@@ -1337,149 +1400,228 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="B43" s="4"/>
-      <c r="C43" s="4"/>
-      <c r="D43" s="4"/>
-      <c r="E43" s="4"/>
+      <c r="B43" s="3"/>
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
         <v>129</v>
       </c>
       <c r="B44" s="1" t="n">
-        <v>36</v>
+        <v>1</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>131</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="2" t="s">
-        <v>131</v>
+      <c r="A45" s="1" t="s">
+        <v>133</v>
       </c>
       <c r="B45" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F45" s="1" t="s">
-        <v>132</v>
+      <c r="C45" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>133</v>
+        <v>60</v>
       </c>
       <c r="B46" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>134</v>
+        <v>6</v>
       </c>
       <c r="B47" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F47" s="1" t="s">
-        <v>132</v>
+      <c r="C47" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B48" s="1" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="B49" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="E49" s="0"/>
-      <c r="F49" s="1" t="s">
-        <v>138</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B50" s="1" t="n">
+      <c r="A50" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
+      <c r="E50" s="4"/>
+    </row>
+    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B51" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B52" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B53" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B54" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B55" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B56" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="E56" s="0"/>
+      <c r="F56" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B57" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C50" s="5" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="6"/>
-      <c r="B51" s="6"/>
-    </row>
-    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="6"/>
-      <c r="B52" s="6"/>
-    </row>
-    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="6"/>
-      <c r="B53" s="6"/>
-    </row>
-    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="6"/>
-      <c r="B54" s="6"/>
-    </row>
-    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="6"/>
-      <c r="B55" s="6"/>
-    </row>
-    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="6"/>
-      <c r="B56" s="6"/>
-    </row>
-    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="6"/>
-      <c r="B57" s="6"/>
+      <c r="C57" s="5" t="s">
+        <v>153</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="6"/>
       <c r="B58" s="6"/>
-      <c r="C58" s="6"/>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="6"/>
       <c r="B59" s="6"/>
-      <c r="C59" s="6"/>
+    </row>
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="6"/>
+      <c r="B60" s="6"/>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="6"/>
+      <c r="B61" s="6"/>
+    </row>
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="6"/>
+      <c r="B62" s="6"/>
+    </row>
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="6"/>
+      <c r="B63" s="6"/>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="2"/>
+      <c r="A64" s="6"/>
+      <c r="B64" s="6"/>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="2"/>
+      <c r="A65" s="6"/>
+      <c r="B65" s="6"/>
+      <c r="C65" s="6"/>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="2"/>
-    </row>
-    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="2"/>
-    </row>
-    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="2"/>
+      <c r="A66" s="6"/>
+      <c r="B66" s="6"/>
+      <c r="C66" s="6"/>
+    </row>
+    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="2"/>
+    </row>
+    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="2"/>
+    </row>
+    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="2"/>
+    </row>
+    <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="2"/>
+    </row>
+    <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A38:E38"/>
     <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A50:E50"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C50" r:id="rId1" display="https://aliexpress.com/item/32896689725.html"/>
+    <hyperlink ref="C57" r:id="rId1" display="https://aliexpress.com/item/32896689725.html"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>